<commit_message>
Ajout des différentes recherches
Ajout composant + list mat, ajout datasheet, ajout images
</commit_message>
<xml_diff>
--- a/Documents/HoferL - JournalPlanif - M7.xlsx
+++ b/Documents/HoferL - JournalPlanif - M7.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>date</t>
   </si>
@@ -126,7 +126,13 @@
     <t>Présentation</t>
   </si>
   <si>
+    <t xml:space="preserve">Recherche des composant chez distributeur</t>
+  </si>
+  <si>
     <t>Somme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Création d'une liste de composant avec prix</t>
   </si>
   <si>
     <t xml:space="preserve">Temps restant </t>
@@ -1664,15 +1670,6 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1680,6 +1677,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="168" xfId="0" applyNumberFormat="1"/>
@@ -4599,8 +4605,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E9">
-  <autoFilter ref="B2:E9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E11">
+  <autoFilter ref="B2:E11"/>
   <tableColumns count="4">
     <tableColumn id="1" name="date" dataDxfId="0"/>
     <tableColumn id="2" name="Temps" dataDxfId="1"/>
@@ -5197,7 +5203,7 @@
       </c>
       <c r="I4" s="11">
         <f>types[[#This Row],[somme]]/$H$10</f>
-        <v>0.11904761904761904</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="13"/>
@@ -5220,11 +5226,11 @@
       </c>
       <c r="H5" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>3.4999999999999996</v>
+        <v>5.9999999999999991</v>
       </c>
       <c r="I5" s="11">
         <f>types[[#This Row],[somme]]/$H$10</f>
-        <v>0.16666666666666666</v>
+        <v>0.24999999999999997</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="13"/>
@@ -5247,11 +5253,11 @@
       </c>
       <c r="H6" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="I6" s="11">
         <f>types[[#This Row],[somme]]/$H$10</f>
-        <v>0.7142857142857143</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="13"/>
@@ -5284,16 +5290,16 @@
       <c r="K7" s="13"/>
     </row>
     <row r="8" ht="28.5">
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="6">
-        <v>0.0625</v>
-      </c>
-      <c r="D8" s="15" t="s">
+        <v>0.125</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G8" s="9" t="s">
@@ -5311,22 +5317,22 @@
       <c r="K8" s="13"/>
     </row>
     <row r="9">
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="6">
         <v>0.125</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="15">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
         <v>0</v>
       </c>
@@ -5335,19 +5341,27 @@
         <v>0</v>
       </c>
       <c r="J9" s="4"/>
-      <c r="K9" s="19"/>
+      <c r="K9" s="16"/>
     </row>
     <row r="10">
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8"/>
+      <c r="B10" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.041666666666666664</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>23</v>
+      </c>
       <c r="G10" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H10" s="10">
         <f>SUM(H3:H9)</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I10" s="11">
         <f>types[[#This Row],[somme]]/$H$10</f>
@@ -5357,10 +5371,18 @@
       <c r="K10" s="4"/>
     </row>
     <row r="11" ht="28.5">
-      <c r="B11" s="5"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8"/>
+      <c r="B11" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.020833333333333332</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>25</v>
+      </c>
       <c r="H11" s="10"/>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -5371,11 +5393,11 @@
       <c r="D12" s="7"/>
       <c r="E12" s="8"/>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H12" s="10">
         <f>SUM(Plannification!C2:S2)-H10</f>
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" ht="42.75">
@@ -5805,13 +5827,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{0025001D-007C-4000-8E90-00BB00850032}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00AB00E0-0001-4D04-93E1-00A4001C0040}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
           <xm:sqref>D8:D55</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00D7006A-002D-4CFE-8984-004900140053}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00210008-00AD-44E6-9F69-001400A400C0}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$9</xm:f>
           </x14:formula1>
@@ -5887,7 +5909,7 @@
       </c>
       <c r="B5" s="27">
         <f>SUMIF(Journal[date],SommeParJours!A5,Journal[Temps])</f>
-        <v>0.1875</v>
+        <v>0.3125</v>
       </c>
       <c r="C5"/>
     </row>
@@ -7540,10 +7562,10 @@
   <sheetData>
     <row r="1" s="32" customFormat="1" ht="66.599999999999994" customHeight="1">
       <c r="A1" s="33" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="35" t="s">
         <v>5</v>
@@ -7555,46 +7577,46 @@
         <v>12</v>
       </c>
       <c r="F1" s="35" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="K1" s="35" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L1" s="35" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="M1" s="35" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N1" s="35" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O1" s="35" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="P1" s="35" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q1" s="35" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="R1" s="35" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="S1" s="35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="T1" s="37"/>
       <c r="U1" s="37"/>
@@ -7635,7 +7657,7 @@
     </row>
     <row r="2" s="32" customFormat="1" ht="16.5" customHeight="1">
       <c r="A2" s="33" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="35">
@@ -7728,10 +7750,10 @@
     </row>
     <row r="3" s="32" customFormat="1" ht="16.5" customHeight="1">
       <c r="A3" s="38" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C3" s="40" t="str">
         <f>_xlfn.CONCAT("Conception Matérielle (",SUM(C2:G2),"h)")</f>
@@ -7821,10 +7843,10 @@
       <c r="R4" s="47"/>
       <c r="S4" s="51"/>
       <c r="V4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W4" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" ht="10.5" customHeight="1">
@@ -7851,7 +7873,7 @@
     <row r="6" ht="10.5" customHeight="1">
       <c r="A6" s="52"/>
       <c r="B6" s="60" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C6" s="61"/>
       <c r="D6" s="62"/>
@@ -7939,7 +7961,7 @@
     <row r="10" ht="10.5" customHeight="1">
       <c r="A10" s="52"/>
       <c r="B10" s="70" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C10" s="62"/>
       <c r="D10" s="61"/>
@@ -7982,10 +8004,10 @@
     </row>
     <row r="12" ht="10.5" customHeight="1">
       <c r="A12" s="82" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B12" s="83" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="46"/>
@@ -8029,7 +8051,7 @@
     <row r="14" ht="10.5" customHeight="1">
       <c r="A14" s="84"/>
       <c r="B14" s="70" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C14" s="62"/>
       <c r="D14" s="61"/>
@@ -8073,7 +8095,7 @@
     <row r="16" ht="10.5" customHeight="1">
       <c r="A16" s="84"/>
       <c r="B16" s="68" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C16" s="55"/>
       <c r="D16" s="61"/>
@@ -8117,7 +8139,7 @@
     <row r="18" ht="10.5" customHeight="1">
       <c r="A18" s="84"/>
       <c r="B18" s="70" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C18" s="62"/>
       <c r="D18" s="62"/>
@@ -8160,10 +8182,10 @@
     </row>
     <row r="20" ht="10.5" customHeight="1">
       <c r="A20" s="44" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B20" s="83" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C20" s="47"/>
       <c r="D20" s="47"/>
@@ -8207,7 +8229,7 @@
     <row r="22" ht="10.5" customHeight="1">
       <c r="A22" s="52"/>
       <c r="B22" s="70" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C22" s="62"/>
       <c r="D22" s="62"/>
@@ -8251,7 +8273,7 @@
     <row r="24" ht="10.5" customHeight="1">
       <c r="A24" s="52"/>
       <c r="B24" s="68" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C24" s="55"/>
       <c r="D24" s="55"/>
@@ -8295,7 +8317,7 @@
     <row r="26" ht="10.5" customHeight="1">
       <c r="A26" s="52"/>
       <c r="B26" s="70" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C26" s="62"/>
       <c r="D26" s="62"/>
@@ -8339,7 +8361,7 @@
     <row r="28" ht="10.5" customHeight="1">
       <c r="A28" s="52"/>
       <c r="B28" s="68" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C28" s="55"/>
       <c r="D28" s="55"/>
@@ -8382,10 +8404,10 @@
     </row>
     <row r="30" ht="10.5" customHeight="1">
       <c r="A30" s="93" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B30" s="94" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C30" s="95"/>
       <c r="D30" s="95"/>
@@ -8429,7 +8451,7 @@
     <row r="32" ht="10.5" customHeight="1">
       <c r="A32" s="99"/>
       <c r="B32" s="70" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C32" s="55"/>
       <c r="D32" s="55"/>
@@ -8473,7 +8495,7 @@
     <row r="34" ht="10.5" customHeight="1">
       <c r="A34" s="99"/>
       <c r="B34" s="70" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C34" s="62"/>
       <c r="D34" s="62"/>
@@ -8517,7 +8539,7 @@
     <row r="36" ht="10.5" customHeight="1">
       <c r="A36" s="99"/>
       <c r="B36" s="68" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C36" s="55"/>
       <c r="D36" s="55"/>
@@ -8561,7 +8583,7 @@
     <row r="38" ht="10.5" customHeight="1">
       <c r="A38" s="99"/>
       <c r="B38" s="70" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C38" s="62"/>
       <c r="D38" s="62"/>
@@ -8605,7 +8627,7 @@
     <row r="40" ht="10.5" customHeight="1">
       <c r="A40" s="99"/>
       <c r="B40" s="68" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C40" s="55"/>
       <c r="D40" s="55"/>
@@ -8649,7 +8671,7 @@
     <row r="42" ht="10.5" customHeight="1">
       <c r="A42" s="99"/>
       <c r="B42" s="70" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C42" s="62"/>
       <c r="D42" s="62"/>
@@ -8692,7 +8714,7 @@
     </row>
     <row r="44" ht="10.5" customHeight="1">
       <c r="A44" s="44" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B44" s="45" t="s">
         <v>22</v>
@@ -8736,14 +8758,14 @@
       <c r="R45" s="55"/>
       <c r="S45" s="59"/>
       <c r="V45" s="102" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="W45" s="61"/>
     </row>
     <row r="46" ht="10.5" customHeight="1">
       <c r="A46" s="52"/>
       <c r="B46" s="103" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C46" s="62"/>
       <c r="D46" s="62"/>
@@ -8763,7 +8785,7 @@
       <c r="R46" s="62"/>
       <c r="S46" s="73"/>
       <c r="V46" s="102" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="W46" s="54"/>
     </row>
@@ -8788,7 +8810,7 @@
       <c r="R47" s="76"/>
       <c r="S47" s="81"/>
       <c r="V47" s="102" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="W47" s="67"/>
     </row>
@@ -8797,7 +8819,7 @@
         <v>46185</v>
       </c>
       <c r="W54" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55" ht="14.25">
@@ -8805,7 +8827,7 @@
         <v>17</v>
       </c>
       <c r="W55" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" ht="14.25">
@@ -8813,7 +8835,7 @@
         <v>18</v>
       </c>
       <c r="W56" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -8881,37 +8903,37 @@
     </row>
     <row r="2" ht="56.399999999999999" customHeight="1">
       <c r="B2" s="107" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="108" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" s="109" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E2" s="110" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F2" s="111" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G2" s="111"/>
       <c r="H2" s="111"/>
       <c r="I2" s="110"/>
       <c r="J2" s="111" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K2" s="111"/>
       <c r="L2" s="111"/>
       <c r="M2" s="110"/>
       <c r="N2" s="111" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O2" s="111"/>
       <c r="P2" s="111"/>
       <c r="Q2" s="110"/>
       <c r="R2" s="111" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="S2" s="112"/>
       <c r="AD2" s="30"/>
@@ -8920,7 +8942,7 @@
       <c r="B3" s="113"/>
       <c r="C3" s="114"/>
       <c r="D3" s="115" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E3" s="116">
         <v>4</v>
@@ -8968,15 +8990,15 @@
         <v>2</v>
       </c>
       <c r="U3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="120" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="108" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D4" s="121"/>
       <c r="E4" s="122"/>
@@ -8995,7 +9017,7 @@
       <c r="R4" s="125"/>
       <c r="S4" s="126"/>
       <c r="U4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -9021,7 +9043,7 @@
     <row r="6" ht="12" customHeight="1">
       <c r="B6" s="120"/>
       <c r="C6" s="135" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D6" s="136"/>
       <c r="E6" s="137"/>
@@ -9040,7 +9062,7 @@
       <c r="R6" s="141"/>
       <c r="S6" s="142"/>
       <c r="U6" s="143" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="V6" s="143"/>
     </row>
@@ -9064,13 +9086,13 @@
       <c r="R7" s="133"/>
       <c r="S7" s="134"/>
       <c r="U7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="120"/>
       <c r="C8" s="135" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D8" s="136"/>
       <c r="E8" s="137"/>
@@ -9089,7 +9111,7 @@
       <c r="R8" s="141"/>
       <c r="S8" s="142"/>
       <c r="U8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -9115,7 +9137,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="120"/>
       <c r="C10" s="135" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D10" s="136"/>
       <c r="E10" s="137"/>
@@ -9156,10 +9178,10 @@
     </row>
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="107" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C12" s="108" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D12" s="121"/>
       <c r="E12" s="122"/>
@@ -9201,7 +9223,7 @@
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="120"/>
       <c r="C14" s="135" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D14" s="154"/>
       <c r="E14" s="137"/>
@@ -9243,7 +9265,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="120"/>
       <c r="C16" s="135" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D16" s="136"/>
       <c r="E16" s="137"/>
@@ -9284,10 +9306,10 @@
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="109" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C18" s="108" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D18" s="121"/>
       <c r="E18" s="122"/>
@@ -9329,7 +9351,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="120"/>
       <c r="C20" s="135" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D20" s="136"/>
       <c r="E20" s="137"/>
@@ -9371,7 +9393,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="120"/>
       <c r="C22" s="135" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D22" s="136"/>
       <c r="E22" s="137"/>
@@ -9412,10 +9434,10 @@
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="109" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C24" s="108" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D24" s="121"/>
       <c r="E24" s="122"/>
@@ -9457,7 +9479,7 @@
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="120"/>
       <c r="C26" s="135" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D26" s="136"/>
       <c r="E26" s="137"/>
@@ -9499,7 +9521,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="120"/>
       <c r="C28" s="135" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D28" s="136"/>
       <c r="E28" s="137"/>
@@ -9543,7 +9565,7 @@
         <v>6</v>
       </c>
       <c r="C30" s="167" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D30" s="121"/>
       <c r="E30" s="168"/>
@@ -9627,7 +9649,7 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="173"/>
       <c r="C34" s="127" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D34" s="159"/>
       <c r="E34" s="187"/>
@@ -9647,7 +9669,7 @@
       <c r="S34" s="191"/>
       <c r="U34" s="192"/>
       <c r="V34" s="193" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" ht="13.800000000000001" customHeight="1">
@@ -9671,7 +9693,7 @@
       <c r="S35" s="151"/>
       <c r="U35" s="200"/>
       <c r="V35" s="201" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout des choix pour le software
</commit_message>
<xml_diff>
--- a/Documents/HoferL - JournalPlanif - M7.xlsx
+++ b/Documents/HoferL - JournalPlanif - M7.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>date</t>
   </si>
@@ -165,10 +165,16 @@
     <t xml:space="preserve">Documentation de l'implémentation du prototypage</t>
   </si>
   <si>
-    <t xml:space="preserve">Discution avec JT (ELT2) pour l'impression de la carte</t>
+    <t xml:space="preserve">Discution avec JET (ELT2) pour l'impression de la carte</t>
   </si>
   <si>
     <t xml:space="preserve">Correction de la violation de la RDC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recherche de solution pour le software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentation des différents choix pour le software</t>
   </si>
   <si>
     <t>Phases</t>
@@ -1720,10 +1726,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -4668,8 +4674,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E21">
-  <autoFilter ref="B2:E21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E23">
+  <autoFilter ref="B2:E23"/>
   <tableColumns count="4">
     <tableColumn id="1" name="date" dataDxfId="0"/>
     <tableColumn id="2" name="Temps" dataDxfId="1"/>
@@ -5266,7 +5272,7 @@
       </c>
       <c r="I4" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>5.1194539249146756e-002</v>
+        <v>4.7318611987381708e-002</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="13"/>
@@ -5289,11 +5295,11 @@
       </c>
       <c r="H5" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>5.9999999999999991</v>
+        <v>7.5</v>
       </c>
       <c r="I5" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.1228668941979522</v>
+        <v>0.14195583596214512</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="13"/>
@@ -5316,11 +5322,11 @@
       </c>
       <c r="H6" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>19.333333333333336</v>
+        <v>21.833333333333332</v>
       </c>
       <c r="I6" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.39590443686006827</v>
+        <v>0.41324921135646692</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="13"/>
@@ -5374,7 +5380,7 @@
       </c>
       <c r="I8" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>2.0477815699658702e-002</v>
+        <v>1.8927444794952682e-002</v>
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="13"/>
@@ -5448,7 +5454,7 @@
       </c>
       <c r="H11" s="10">
         <f>SUM(H3:H10)</f>
-        <v>48.833333333333336</v>
+        <v>52.833333333333329</v>
       </c>
       <c r="I11" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
@@ -5492,7 +5498,7 @@
       </c>
       <c r="H13" s="10">
         <f>SUM(Plannification!C2:S2)-H11</f>
-        <v>26.166666666666664</v>
+        <v>22.166666666666671</v>
       </c>
     </row>
     <row r="14" ht="42.75">
@@ -5586,10 +5592,10 @@
       <c r="C20" s="6">
         <v>6.25e-002</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="18" t="s">
         <v>36</v>
       </c>
     </row>
@@ -5603,21 +5609,37 @@
       <c r="D21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="5"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="8"/>
+      <c r="B22" s="5">
+        <v>46149</v>
+      </c>
+      <c r="C22" s="6">
+        <v>6.25e-002</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="23">
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="8"/>
+      <c r="B23" s="5">
+        <v>46149</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="5"/>
@@ -5986,13 +6008,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{003600E8-006D-4CC2-9228-00AA001F0084}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00EE005C-00CC-4422-A291-00F800DA001D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$11</xm:f>
           </x14:formula1>
           <xm:sqref>D8 D13:D56 D11 D12</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00940001-00B5-4FBA-AB6C-005300D1007A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{003300C3-00C7-467E-9229-00B200B000A4}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
@@ -6112,7 +6134,7 @@
       </c>
       <c r="B9" s="27">
         <f>SUMIF(Journal[date],SommeParJours!A9,Journal[Temps])</f>
-        <v>0.18749999999999997</v>
+        <v>0.35416666666666663</v>
       </c>
       <c r="C9"/>
     </row>
@@ -7733,10 +7755,10 @@
   <sheetData>
     <row r="1" s="32" customFormat="1" ht="66.599999999999994" customHeight="1">
       <c r="A1" s="33" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C1" s="35" t="s">
         <v>5</v>
@@ -7748,46 +7770,46 @@
         <v>12</v>
       </c>
       <c r="F1" s="35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K1" s="35" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="L1" s="35" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="M1" s="35" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N1" s="35" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O1" s="35" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="P1" s="35" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="Q1" s="35" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="R1" s="35" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="S1" s="35" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="T1" s="37"/>
       <c r="U1" s="37"/>
@@ -7828,7 +7850,7 @@
     </row>
     <row r="2" s="32" customFormat="1" ht="16.5" customHeight="1">
       <c r="A2" s="33" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="35">
@@ -7921,10 +7943,10 @@
     </row>
     <row r="3" s="32" customFormat="1" ht="16.5" customHeight="1">
       <c r="A3" s="38" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="40" t="str">
         <f>_xlfn.CONCAT("Conception Matérielle (",SUM(C2:G2),"h)")</f>
@@ -8017,10 +8039,10 @@
       <c r="R4" s="48"/>
       <c r="S4" s="52"/>
       <c r="V4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="W4" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" ht="10.5" customHeight="1">
@@ -8047,7 +8069,7 @@
     <row r="6" ht="10.5" customHeight="1">
       <c r="A6" s="53"/>
       <c r="B6" s="61" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C6" s="62"/>
       <c r="D6" s="63"/>
@@ -8135,7 +8157,7 @@
     <row r="10" ht="10.5" customHeight="1">
       <c r="A10" s="53"/>
       <c r="B10" s="71" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C10" s="63"/>
       <c r="D10" s="62"/>
@@ -8178,10 +8200,10 @@
     </row>
     <row r="12" ht="10.5" customHeight="1">
       <c r="A12" s="83" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="84" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="47"/>
@@ -8225,7 +8247,7 @@
     <row r="14" ht="10.5" customHeight="1">
       <c r="A14" s="85"/>
       <c r="B14" s="71" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C14" s="63"/>
       <c r="D14" s="62"/>
@@ -8269,7 +8291,7 @@
     <row r="16" ht="10.5" customHeight="1">
       <c r="A16" s="85"/>
       <c r="B16" s="69" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C16" s="56"/>
       <c r="D16" s="62"/>
@@ -8313,7 +8335,7 @@
     <row r="18" ht="10.5" customHeight="1">
       <c r="A18" s="85"/>
       <c r="B18" s="71" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C18" s="63"/>
       <c r="D18" s="63"/>
@@ -8356,10 +8378,10 @@
     </row>
     <row r="20" ht="10.5" customHeight="1">
       <c r="A20" s="45" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B20" s="84" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C20" s="48"/>
       <c r="D20" s="48"/>
@@ -8403,7 +8425,7 @@
     <row r="22" ht="10.5" customHeight="1">
       <c r="A22" s="53"/>
       <c r="B22" s="71" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C22" s="63"/>
       <c r="D22" s="63"/>
@@ -8447,7 +8469,7 @@
     <row r="24" ht="10.5" customHeight="1">
       <c r="A24" s="53"/>
       <c r="B24" s="69" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C24" s="56"/>
       <c r="D24" s="56"/>
@@ -8491,7 +8513,7 @@
     <row r="26" ht="10.5" customHeight="1">
       <c r="A26" s="53"/>
       <c r="B26" s="71" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C26" s="63"/>
       <c r="D26" s="63"/>
@@ -8535,7 +8557,7 @@
     <row r="28" ht="10.5" customHeight="1">
       <c r="A28" s="53"/>
       <c r="B28" s="69" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C28" s="56"/>
       <c r="D28" s="56"/>
@@ -8578,10 +8600,10 @@
     </row>
     <row r="30" ht="10.5" customHeight="1">
       <c r="A30" s="96" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B30" s="97" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C30" s="98"/>
       <c r="D30" s="98"/>
@@ -8625,7 +8647,7 @@
     <row r="32" ht="10.5" customHeight="1">
       <c r="A32" s="102"/>
       <c r="B32" s="71" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C32" s="56"/>
       <c r="D32" s="56"/>
@@ -8669,7 +8691,7 @@
     <row r="34" ht="10.5" customHeight="1">
       <c r="A34" s="102"/>
       <c r="B34" s="71" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C34" s="63"/>
       <c r="D34" s="63"/>
@@ -8713,7 +8735,7 @@
     <row r="36" ht="10.5" customHeight="1">
       <c r="A36" s="102"/>
       <c r="B36" s="69" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C36" s="56"/>
       <c r="D36" s="56"/>
@@ -8757,7 +8779,7 @@
     <row r="38" ht="10.5" customHeight="1">
       <c r="A38" s="102"/>
       <c r="B38" s="71" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C38" s="63"/>
       <c r="D38" s="63"/>
@@ -8801,7 +8823,7 @@
     <row r="40" ht="10.5" customHeight="1">
       <c r="A40" s="102"/>
       <c r="B40" s="69" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C40" s="56"/>
       <c r="D40" s="56"/>
@@ -8845,7 +8867,7 @@
     <row r="42" ht="10.5" customHeight="1">
       <c r="A42" s="102"/>
       <c r="B42" s="71" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C42" s="63"/>
       <c r="D42" s="63"/>
@@ -8888,7 +8910,7 @@
     </row>
     <row r="44" ht="10.5" customHeight="1">
       <c r="A44" s="45" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B44" s="46" t="s">
         <v>24</v>
@@ -8932,14 +8954,14 @@
       <c r="R45" s="56"/>
       <c r="S45" s="60"/>
       <c r="V45" s="105" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="W45" s="62"/>
     </row>
     <row r="46" ht="10.5" customHeight="1">
       <c r="A46" s="53"/>
       <c r="B46" s="106" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C46" s="63"/>
       <c r="D46" s="63"/>
@@ -8959,7 +8981,7 @@
       <c r="R46" s="63"/>
       <c r="S46" s="74"/>
       <c r="V46" s="105" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="W46" s="55"/>
     </row>
@@ -8984,7 +9006,7 @@
       <c r="R47" s="77"/>
       <c r="S47" s="82"/>
       <c r="V47" s="105" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="W47" s="68"/>
     </row>
@@ -8993,7 +9015,7 @@
         <v>46185</v>
       </c>
       <c r="W54" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" ht="14.25">
@@ -9001,7 +9023,7 @@
         <v>17</v>
       </c>
       <c r="W55" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" ht="14.25">
@@ -9009,7 +9031,7 @@
         <v>18</v>
       </c>
       <c r="W56" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -9077,37 +9099,37 @@
     </row>
     <row r="2" ht="56.399999999999999" customHeight="1">
       <c r="B2" s="110" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="111" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" s="112" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="113" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="114" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="114"/>
       <c r="H2" s="114"/>
       <c r="I2" s="113"/>
       <c r="J2" s="114" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K2" s="114"/>
       <c r="L2" s="114"/>
       <c r="M2" s="113"/>
       <c r="N2" s="114" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="O2" s="114"/>
       <c r="P2" s="114"/>
       <c r="Q2" s="113"/>
       <c r="R2" s="114" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="S2" s="115"/>
       <c r="AD2" s="30"/>
@@ -9116,7 +9138,7 @@
       <c r="B3" s="116"/>
       <c r="C3" s="117"/>
       <c r="D3" s="118" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" s="119">
         <v>4</v>
@@ -9164,15 +9186,15 @@
         <v>2</v>
       </c>
       <c r="U3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="123" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C4" s="111" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D4" s="124"/>
       <c r="E4" s="125"/>
@@ -9191,7 +9213,7 @@
       <c r="R4" s="128"/>
       <c r="S4" s="129"/>
       <c r="U4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -9217,7 +9239,7 @@
     <row r="6" ht="12" customHeight="1">
       <c r="B6" s="123"/>
       <c r="C6" s="138" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D6" s="139"/>
       <c r="E6" s="140"/>
@@ -9236,7 +9258,7 @@
       <c r="R6" s="144"/>
       <c r="S6" s="145"/>
       <c r="U6" s="146" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="V6" s="146"/>
     </row>
@@ -9260,13 +9282,13 @@
       <c r="R7" s="136"/>
       <c r="S7" s="137"/>
       <c r="U7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="123"/>
       <c r="C8" s="138" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D8" s="139"/>
       <c r="E8" s="140"/>
@@ -9285,7 +9307,7 @@
       <c r="R8" s="144"/>
       <c r="S8" s="145"/>
       <c r="U8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -9311,7 +9333,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="123"/>
       <c r="C10" s="138" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D10" s="139"/>
       <c r="E10" s="140"/>
@@ -9352,10 +9374,10 @@
     </row>
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="110" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C12" s="111" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D12" s="124"/>
       <c r="E12" s="125"/>
@@ -9397,7 +9419,7 @@
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="123"/>
       <c r="C14" s="138" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D14" s="157"/>
       <c r="E14" s="140"/>
@@ -9439,7 +9461,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="123"/>
       <c r="C16" s="138" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D16" s="139"/>
       <c r="E16" s="140"/>
@@ -9480,10 +9502,10 @@
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="112" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C18" s="111" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D18" s="124"/>
       <c r="E18" s="125"/>
@@ -9525,7 +9547,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="123"/>
       <c r="C20" s="138" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D20" s="139"/>
       <c r="E20" s="140"/>
@@ -9567,7 +9589,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="123"/>
       <c r="C22" s="138" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D22" s="139"/>
       <c r="E22" s="140"/>
@@ -9608,10 +9630,10 @@
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="112" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C24" s="111" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D24" s="124"/>
       <c r="E24" s="125"/>
@@ -9653,7 +9675,7 @@
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="123"/>
       <c r="C26" s="138" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D26" s="139"/>
       <c r="E26" s="140"/>
@@ -9695,7 +9717,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="123"/>
       <c r="C28" s="138" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D28" s="139"/>
       <c r="E28" s="140"/>
@@ -9739,7 +9761,7 @@
         <v>6</v>
       </c>
       <c r="C30" s="170" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D30" s="124"/>
       <c r="E30" s="171"/>
@@ -9823,7 +9845,7 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="176"/>
       <c r="C34" s="130" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D34" s="162"/>
       <c r="E34" s="190"/>
@@ -9843,7 +9865,7 @@
       <c r="S34" s="194"/>
       <c r="U34" s="195"/>
       <c r="V34" s="196" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" ht="13.800000000000001" customHeight="1">
@@ -9867,7 +9889,7 @@
       <c r="S35" s="154"/>
       <c r="U35" s="203"/>
       <c r="V35" s="204" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>